<commit_message>
Rà soát bộ mẫu cấp 1–2: thống nhất dữ liệu mẫu giữa các văn bản, sửa trích TCVN nhật ký, ngày ký kế hoạch
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EYfrLZFALxho7iwpK7bTVa
</commit_message>
<xml_diff>
--- a/templates/08-bo-mau-cap-1-2/checklist-cap-1-2.xlsx
+++ b/templates/08-bo-mau-cap-1-2/checklist-cap-1-2.xlsx
@@ -8974,7 +8974,7 @@
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="22.7" customWidth="1" min="6" max="6"/>
-    <col width="30.8" customWidth="1" min="7" max="7"/>
+    <col width="34.4" customWidth="1" min="7" max="7"/>
     <col width="27.2" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -9067,12 +9067,12 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>31/03/2027</t>
+          <t>31/12/2026 (theo QĐ 03/2026/QĐ-PANM)</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>Đang thực hiện</t>
+          <t>Đã hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bộ cấp 1–2: 7 mẫu bảo vệ DLCN, kiểm kê DLCN; đối chiếu văn bản dẫn chiếu ngoài
- Mẫu 10–16: thông báo xử lý DLCN cho người lao động, ứng viên; phiếu đồng ý;
  quy trình yêu cầu của chủ thể dữ liệu; cam kết bảo mật của nhân sự; phụ lục
  hợp đồng BVDLCN với bên xử lý/cloud; biển báo camera (Word, dữ liệu mẫu)
- Bảng tính cấp 1–2: sheet F kiểm kê dữ liệu cá nhân
- danh-muc-van-ban mục 3a: BLLĐ 2019 Đ21.2, 118–119, 124, 125.2, 129; BLHS Đ159,
  288.1.b, 289.1 (tội riêng về DLCN mới là dự thảo); Luật 04/2017 Đ3.2, Đ4;
  NĐ 80/2021 Đ5; NĐ 30/2020 Đ2.1; Luật Doanh nghiệp 2020 Đ43 — đối chiếu qua
  nguồn thứ cấp, chưa có toàn văn
- Gỡ [CẦN ĐỐI CHIẾU] đã xác nhận ở mẫu 14, Mẫu 01, trang BVDLCN (bảng tiêu chí DN
  siêu nhỏ, nhỏ theo NĐ 80/2021)
- Cập nhật mục lục: docs/08 README, templates/README, README gốc (49 Word), en/08,
  en/09 (54 file)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EYfrLZFALxho7iwpK7bTVa
</commit_message>
<xml_diff>
--- a/templates/08-bo-mau-cap-1-2/checklist-cap-1-2.xlsx
+++ b/templates/08-bo-mau-cap-1-2/checklist-cap-1-2.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C. Lịch định kỳ" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D. Sổ sự cố" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E. Kế hoạch khắc phục" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F. Kiểm kê DLCN" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'A. Danh mục HTTT'!$A$4:$H$18</definedName>
@@ -26,6 +27,8 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'D. Sổ sự cố'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'E. Kế hoạch khắc phục'!$A$4:$H$37</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'E. Kế hoạch khắc phục'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'F. Kiểm kê DLCN'!$A$4:$K$32</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'F. Kiểm kê DLCN'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9465,4 +9468,820 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:K32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>F. KIỂM KÊ DỮ LIỆU CÁ NHÂN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Hàng mẫu mô phỏng. Nhạy cảm theo NĐ 356 Đ4.1; dùng làm đầu vào cho DPIA, hồ sơ chuyển xuyên biên giới và xác định miễn trừ DN nhỏ (Luật 91 Đ38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>HTTT / quy trình</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Nhóm chủ thể</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Loại DLCN</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Cơ bản / Nhạy cảm (NĐ 356 Đ4.1)</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Mục đích</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Căn cứ xử lý</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Số chủ thể (ước tính)</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Nơi lưu (VN/nước ngoài, nhà cung cấp)</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Bên nhận</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Thời hạn lưu</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Người phụ trách</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Tuyển dụng — hộp thư tuyển dụng (HT-02-INTRANET), phân hệ nhân sự (HT-03-ERP)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Ứng viên</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Họ tên, ngày sinh, điện thoại, email, CV, bằng cấp, kinh nghiệm, ảnh chân dung</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Cơ bản (NĐ 356 Đ3)</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Tuyển dụng; nguồn ứng viên nếu ứng viên đồng ý</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Đồng ý của ứng viên (Luật 91 Đ25.1.b) — Thông báo ứng viên (mẫu 11)</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>~300/năm</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>VN — ERP tại phòng máy trụ sở; hộp thư trên cloud của Công ty TNHH Dữ liệu Mẫu (máy chủ TP. Hồ Chí Minh)</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Không chuyển cho bên ngoài; Công ty TNHH Dữ liệu Mẫu là bên xử lý (phụ lục PL-01)</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>Không trúng tuyển: xóa sau 30 ngày kể từ khi thông báo kết quả; nguồn ứng viên: 12 tháng (Luật 91 Đ25.1.c)</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Phòng Hành chính – Nhân sự</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Hồ sơ nhân sự — HT-03-ERP (phân hệ nhân sự), tủ hồ sơ giấy</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Người lao động; người thân khai để liên hệ, giảm trừ gia cảnh</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Họ tên, ngày sinh, số CCCD, địa chỉ, quan hệ gia đình, hợp đồng lao động, trình độ; ảnh thẻ căn cước chỉ khi hồ sơ bảo hiểm xã hội yêu cầu</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Cơ bản; ảnh thẻ căn cước: nhạy cảm (Đ4.1.i) — lưu tách riêng, mã hóa</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Quản lý lao động</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Thực hiện hợp đồng lao động (Luật 91 Đ19.1.d); ảnh thẻ căn cước: đồng ý (mẫu 12)</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>120 NLĐ; ~150 người thân</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>VN — ERP tại phòng máy Tầng 3</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan nhà nước khi có yêu cầu bằng văn bản; Công ty TNHH Phần mềm Mẫu (bảo trì ERP — bên xử lý)</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Thời gian làm việc + 12 tháng sau nghỉ việc; ảnh thẻ căn cước: xóa ngay khi xong thủ tục bảo hiểm xã hội (Luật 91 Đ25.2)</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>Phòng Hành chính – Nhân sự</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Lương, bảo hiểm, thuế — HT-03-ERP (phân hệ kế toán, tiền lương)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Người lao động; người phụ thuộc</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Lương, mã số thuế, số sổ bảo hiểm xã hội, số tài khoản nhận lương; giấy khám sức khỏe, nghỉ ốm, thai sản</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Cơ bản; sức khỏe: nhạy cảm (Đ4.1.d); số tài khoản ngân hàng: chưa rõ (Đ4.1.k) [CẦN ĐỐI CHIẾU]</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Trả lương; đóng bảo hiểm; khấu trừ thuế thu nhập cá nhân; chế độ ốm đau, thai sản</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Hợp đồng lao động (Đ19.1.d); nghĩa vụ luật định (Đ19.1.đ); sức khỏe: Luật 91 Đ26.1.a — đồng ý hoặc Đ19.1 [CẦN ĐỐI CHIẾU]</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>120 NLĐ; ~150 người phụ thuộc</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>VN — ERP tại phòng máy Tầng 3</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan bảo hiểm xã hội; cơ quan thuế; ngân hàng chi lương</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>Theo thời hạn pháp luật kế toán, thuế, bảo hiểm [CẦN ĐỐI CHIẾU]; sức khỏe: xóa khi chấm dứt hợp đồng lao động trừ hồ sơ pháp luật buộc lưu</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>Phòng Tài chính – Kế toán</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Thư điện tử, văn phòng điện tử — HT-02-INTRANET</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Người lao động; khách hàng, đối tác, ứng viên trao đổi thư</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Họ tên, email, chức danh, điện thoại, nội dung thư, tệp đính kèm; nhật ký đăng nhập</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Cơ bản; tệp đính kèm có thể lẫn dữ liệu nhạy cảm</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Điều hành, liên lạc công việc</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Hợp đồng lao động (Đ19.1.d); với người bên ngoài: thực hiện giao dịch, hợp đồng (Đ19.1.d) [CẦN ĐỐI CHIẾU]</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>120 hộp thư; ~2.000 người liên hệ bên ngoài</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>VN — cloud của Công ty TNHH Dữ liệu Mẫu (TP. Hồ Chí Minh; dự phòng Hà Nội); không chuyển ra nước ngoài</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Công ty TNHH Dữ liệu Mẫu (bên xử lý — phụ lục PL-01 kèm HĐ 08/2026/HĐDV/TURBO-DLM)</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Hộp thư của người nghỉ việc: 30 ngày để bàn giao rồi xóa; bản sao lưu: 30 ngày</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>Phòng Vận hành hệ thống</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Danh bạ khách hàng, đối tác — bảng tính dùng chung trên HT-02-INTRANET</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Người liên hệ của khách hàng, đối tác; khách hàng cá nhân</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Họ tên, chức danh, nơi công tác, điện thoại, email, lịch sử giao dịch</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Cơ bản</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Chăm sóc khách hàng, thực hiện hợp đồng</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Thực hiện hợp đồng (Đ19.1.d); người liên hệ của doanh nghiệp đối tác không phải bên hợp đồng [CẦN ĐỐI CHIẾU]</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>~1.500</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>VN — cloud của Công ty TNHH Dữ liệu Mẫu</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>Rà soát hằng năm; xóa người liên hệ không còn giao dịch sau 24 tháng</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Phòng Kinh doanh</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Camera — sảnh lễ tân, cửa ra vào (đầu ghi tại phòng máy)</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Người lao động; khách đến làm việc</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Hình ảnh (không ghi âm, không nhận diện khuôn mặt)</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Cơ bản (hình ảnh — NĐ 356 Đ3.6); bật nhận diện khuôn mặt sẽ thành sinh trắc học nhạy cảm (Đ4.1.đ)</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>An ninh, an toàn người và tài sản</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Luật 91 Đ32.1.a; biển báo (Đ32.2 — mẫu 16); thông báo người lao động (Đ25.3 — mẫu 10)</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>120 NLĐ; ~50 khách/ngày</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>VN — đầu ghi tại trụ sở</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan nhà nước khi có yêu cầu bằng văn bản</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>30 ngày, tự ghi đè (Luật 91 Đ32.4)</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>Phòng Hành chính – Nhân sự</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Chấm công thẻ từ — máy chấm công tại cửa, đồng bộ vào HT-03-ERP</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Người lao động</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Mã thẻ, họ tên, giờ vào, giờ ra</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Cơ bản (không dùng vân tay, khuôn mặt)</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Tính công, tính lương</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Hợp đồng lao động (Đ19.1.d); thông báo biện pháp theo dõi (Đ25.3)</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>VN — máy chấm công và ERP tại trụ sở</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>Theo thời hạn lưu chứng từ tiền lương</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>Phòng Hành chính – Nhân sự</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Tài khoản, nhật ký hệ thống — HT-04-LAN (Active Directory), tường lửa, nhật ký ERP, Intranet</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Người lao động</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Tên tài khoản, nhật ký đăng nhập, thao tác, địa chỉ IP, tên miền truy cập Internet</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Cơ bản; nhật ký theo dõi hành vi sử dụng dịch vụ trên mạng có thể thuộc Đ4.1.l [CẦN ĐỐI CHIẾU]</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Bảo đảm an ninh mạng; điều tra sự cố</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Nghĩa vụ an ninh mạng theo luật (Đ19.1.đ) [CẦN ĐỐI CHIẾU]; thông báo người lao động (Đ25.3)</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>VN — máy chủ nhật ký tại phòng máy Tầng 3</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>06 tháng</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>Phòng Vận hành hệ thống; Phòng An ninh mạng rà soát</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="12" t="n"/>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="12" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="12" t="n"/>
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="12" t="n"/>
+      <c r="J14" s="12" t="n"/>
+      <c r="K14" s="12" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="12" t="n"/>
+      <c r="G15" s="12" t="n"/>
+      <c r="H15" s="12" t="n"/>
+      <c r="I15" s="12" t="n"/>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="12" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="12" t="n"/>
+      <c r="I16" s="12" t="n"/>
+      <c r="J16" s="12" t="n"/>
+      <c r="K16" s="12" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="12" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n"/>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="12" t="n"/>
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="12" t="n"/>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="12" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="12" t="n"/>
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="12" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="12" t="n"/>
+      <c r="I20" s="12" t="n"/>
+      <c r="J20" s="12" t="n"/>
+      <c r="K20" s="12" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n"/>
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="12" t="n"/>
+      <c r="I21" s="12" t="n"/>
+      <c r="J21" s="12" t="n"/>
+      <c r="K21" s="12" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n"/>
+      <c r="B22" s="12" t="n"/>
+      <c r="C22" s="12" t="n"/>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="12" t="n"/>
+      <c r="H22" s="12" t="n"/>
+      <c r="I22" s="12" t="n"/>
+      <c r="J22" s="12" t="n"/>
+      <c r="K22" s="12" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n"/>
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="12" t="n"/>
+      <c r="J23" s="12" t="n"/>
+      <c r="K23" s="12" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n"/>
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="12" t="n"/>
+      <c r="H24" s="12" t="n"/>
+      <c r="I24" s="12" t="n"/>
+      <c r="J24" s="12" t="n"/>
+      <c r="K24" s="12" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n"/>
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="12" t="n"/>
+      <c r="I25" s="12" t="n"/>
+      <c r="J25" s="12" t="n"/>
+      <c r="K25" s="12" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n"/>
+      <c r="B26" s="12" t="n"/>
+      <c r="C26" s="12" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="12" t="n"/>
+      <c r="F26" s="12" t="n"/>
+      <c r="G26" s="12" t="n"/>
+      <c r="H26" s="12" t="n"/>
+      <c r="I26" s="12" t="n"/>
+      <c r="J26" s="12" t="n"/>
+      <c r="K26" s="12" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n"/>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="12" t="n"/>
+      <c r="J27" s="12" t="n"/>
+      <c r="K27" s="12" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n"/>
+      <c r="B28" s="12" t="n"/>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="12" t="n"/>
+      <c r="H28" s="12" t="n"/>
+      <c r="I28" s="12" t="n"/>
+      <c r="J28" s="12" t="n"/>
+      <c r="K28" s="12" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n"/>
+      <c r="B29" s="12" t="n"/>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="12" t="n"/>
+      <c r="H29" s="12" t="n"/>
+      <c r="I29" s="12" t="n"/>
+      <c r="J29" s="12" t="n"/>
+      <c r="K29" s="12" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n"/>
+      <c r="B30" s="12" t="n"/>
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="12" t="n"/>
+      <c r="G30" s="12" t="n"/>
+      <c r="H30" s="12" t="n"/>
+      <c r="I30" s="12" t="n"/>
+      <c r="J30" s="12" t="n"/>
+      <c r="K30" s="12" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n"/>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+      <c r="I31" s="12" t="n"/>
+      <c r="J31" s="12" t="n"/>
+      <c r="K31" s="12" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n"/>
+      <c r="B32" s="12" t="n"/>
+      <c r="C32" s="12" t="n"/>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="12" t="n"/>
+      <c r="F32" s="12" t="n"/>
+      <c r="G32" s="12" t="n"/>
+      <c r="H32" s="12" t="n"/>
+      <c r="I32" s="12" t="n"/>
+      <c r="J32" s="12" t="n"/>
+      <c r="K32" s="12" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:K32"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rà soát mẫu BVDLCN (đợt 2): cam kết 14 bám BLLĐ Đ125.2, Đ129; phụ lục 15 không làm chậm thông báo vi phạm; thống nhất vị trí lưu trữ, thời hạn ảnh CCCD, thuật ngữ tiếng Anh
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EYfrLZFALxho7iwpK7bTVa
</commit_message>
<xml_diff>
--- a/templates/08-bo-mau-cap-1-2/checklist-cap-1-2.xlsx
+++ b/templates/08-bo-mau-cap-1-2/checklist-cap-1-2.xlsx
@@ -9668,7 +9668,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Thời gian làm việc + 12 tháng sau nghỉ việc; ảnh thẻ căn cước: xóa ngay khi xong thủ tục bảo hiểm xã hội (Luật 91 Đ25.2)</t>
+          <t>Thời gian làm việc + 12 tháng sau nghỉ việc; ảnh thẻ căn cước: xóa khi hoàn thành thủ tục bảo hiểm xã hội (chậm nhất khi nghỉ việc), hoặc sớm hơn khi rút lại đồng ý (Luật 91 Đ25.2; NĐ 356 Đ5.2)</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
@@ -9980,7 +9980,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Cơ bản; nhật ký theo dõi hành vi sử dụng dịch vụ trên mạng có thể thuộc Đ4.1.l [CẦN ĐỐI CHIẾU]</t>
+          <t>Cơ bản; nhật ký theo dõi hành vi sử dụng dịch vụ trên mạng (tên miền truy cập Internet) có thể thuộc Đ4.1.l — bảo vệ như dữ liệu nhạy cảm (phân quyền — Đ4.2) [CẦN ĐỐI CHIẾU]</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Bộ cấp 1–2: hoàn thiện hồ sơ BVDLCN (20 DPIA, 21 thông báo vi phạm), xuất Word 17–23, cập nhật danh mục và bản tiếng Anh
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EYfrLZFALxho7iwpK7bTVa
</commit_message>
<xml_diff>
--- a/templates/08-bo-mau-cap-1-2/checklist-cap-1-2.xlsx
+++ b/templates/08-bo-mau-cap-1-2/checklist-cap-1-2.xlsx
@@ -9485,7 +9485,7 @@
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
@@ -9596,7 +9596,7 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>~300/năm</t>
+          <t>~80/năm</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
@@ -9653,7 +9653,7 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>120 NLĐ; ~150 người thân</t>
+          <t>38 NLĐ; ~50 người thân</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -9710,7 +9710,7 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>120 NLĐ; ~150 người phụ thuộc</t>
+          <t>38 NLĐ; ~50 người phụ thuộc</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
@@ -9767,7 +9767,7 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>120 hộp thư; ~2.000 người liên hệ bên ngoài</t>
+          <t>40 hộp thư; ~800 người liên hệ bên ngoài</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -9824,7 +9824,7 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>~1.500</t>
+          <t>~600</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -9881,7 +9881,7 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>120 NLĐ; ~50 khách/ngày</t>
+          <t>38 NLĐ; ~15 khách/ngày</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
@@ -9938,7 +9938,7 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>38</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
@@ -9995,7 +9995,7 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>40</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">

</xml_diff>